<commit_message>
feat: complete income page with chart, filters, export and CRUD operations
</commit_message>
<xml_diff>
--- a/backend/income_details.xlsx
+++ b/backend/income_details.xlsx
@@ -415,16 +415,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Web Project</v>
+        <v>Food</v>
       </c>
       <c r="B2">
-        <v>15000</v>
+        <v>1500</v>
       </c>
       <c r="C2" t="str">
-        <v>Freelancing</v>
+        <v>Food</v>
       </c>
       <c r="D2" t="str">
-        <v>2/9/2026</v>
+        <v>3/17/2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>